<commit_message>
Balance 144-service focus across 18 days
</commit_message>
<xml_diff>
--- a/plan/Plan_Diario_Oficina_Inteligente_JB_144_Servicios.xlsx
+++ b/plan/Plan_Diario_Oficina_Inteligente_JB_144_Servicios.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel mensual" sheetId="1" r:id="R1a675f6acb174314"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda diaria" sheetId="2" r:id="R04790c3a9ede4b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicios" sheetId="3" r:id="Raabd2ed6f4a14f73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel mensual" sheetId="1" r:id="R87ca2d8519bd4c47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda diaria" sheetId="2" r:id="R5e4e8f694e674aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicios" sheetId="3" r:id="Rd3ad3852ea1e499f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1230,16 +1230,16 @@
       </x:c>
       <x:c r="B8" s="24"/>
       <x:c r="C8" s="26" t="str">
-        <x:v>Análisis documental + Archivo privado</x:v>
+        <x:v>Análisis documental</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>11, 12, 13, 14, 15, 16, 23, 24, 25, 26, 27, 28</x:v>
+        <x:v>11, 12, 13, 14, 15, 16</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 11, 12, 13, 14, 15, 16, 23, 24, 25, 26, 27, 28 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 11, 12, 13, 14, 15, 16 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Matriz de hallazgos y comparación · Índice de expediente y reglas de archivo</x:v>
+        <x:v>Matriz de hallazgos y comparación</x:v>
       </x:c>
       <x:c r="G8" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1256,16 +1256,16 @@
       </x:c>
       <x:c r="B9" s="24"/>
       <x:c r="C9" s="26" t="str">
-        <x:v>Control interno + Capital humano</x:v>
+        <x:v>Archivo privado</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>69, 70, 71, 72, 73, 74, 81, 82, 83, 84, 85, 86, 87, 88, 90, 91, 97</x:v>
+        <x:v>23, 24, 25, 26, 27, 28</x:v>
       </x:c>
       <x:c r="E9" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 69, 70, 71, 72, 73, 74, 81, 82, 83, 84, 85, 86, 87, 88, 90, 91, 97 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 23, 24, 25, 26, 27, 28 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F9" s="26" t="str">
-        <x:v>Matriz de controles y plan de medidas · Organigrama, perfiles y controles auxiliares</x:v>
+        <x:v>Índice de expediente y reglas de archivo</x:v>
       </x:c>
       <x:c r="G9" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1282,16 +1282,16 @@
       </x:c>
       <x:c r="B10" s="24"/>
       <x:c r="C10" s="26" t="str">
-        <x:v>Formación y desempeño</x:v>
+        <x:v>Control interno</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
-        <x:v>94, 95</x:v>
+        <x:v>69, 70, 71, 72, 73, 74, 81, 82, 83, 84, 85, 86, 87</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 94, 95 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 69, 70, 71, 72, 73, 74, 81, 82, 83, 84, 85, 86, 87 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>Plan de formación y evaluación</x:v>
+        <x:v>Matriz de controles y plan de medidas</x:v>
       </x:c>
       <x:c r="G10" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1308,16 +1308,16 @@
       </x:c>
       <x:c r="B11" s="24"/>
       <x:c r="C11" s="26" t="str">
-        <x:v>Trabajo y contratos + Seguridad y salud</x:v>
+        <x:v>Capital humano + Formación y desempeño</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>63, 64, 65, 66, 67, 68, 89, 96</x:v>
+        <x:v>88, 90, 91, 94, 95, 97</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 63, 64, 65, 66, 67, 68, 89, 96 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 88, 90, 91, 94, 95, 97 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F11" s="26" t="str">
-        <x:v>Borrador y matriz de obligaciones · Matriz SST y plan preventivo</x:v>
+        <x:v>Organigrama, perfiles y controles auxiliares · Plan de formación y evaluación</x:v>
       </x:c>
       <x:c r="G11" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1334,16 +1334,16 @@
       </x:c>
       <x:c r="B12" s="24"/>
       <x:c r="C12" s="26" t="str">
-        <x:v>Economía y finanzas + Presupuestos y costos</x:v>
+        <x:v>Trabajo y contratos</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
-        <x:v>47, 48, 50, 51, 52, 53, 54, 55</x:v>
+        <x:v>63, 64, 65, 66, 67, 68, 89</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 47, 48, 50, 51, 52, 53, 54, 55 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 63, 64, 65, 66, 67, 68, 89 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
-        <x:v>Análisis y escenarios verificables · Modelo de costos y presupuesto</x:v>
+        <x:v>Borrador y matriz de obligaciones</x:v>
       </x:c>
       <x:c r="G12" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1360,16 +1360,16 @@
       </x:c>
       <x:c r="B13" s="24"/>
       <x:c r="C13" s="26" t="str">
-        <x:v>Factibilidad</x:v>
+        <x:v>Seguridad y salud + Economía y finanzas + Presupuestos y costos</x:v>
       </x:c>
       <x:c r="D13" s="26" t="str">
-        <x:v>56, 104</x:v>
+        <x:v>47, 48, 50, 51, 52, 53, 54, 55, 96</x:v>
       </x:c>
       <x:c r="E13" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 56, 104 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 47, 48, 50, 51, 52, 53, 54, 55, 96 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F13" s="26" t="str">
-        <x:v>Estudio de factibilidad y modelo</x:v>
+        <x:v>Matriz SST y plan preventivo · Análisis y escenarios verificables · Modelo de costos y presupuesto</x:v>
       </x:c>
       <x:c r="G13" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1386,16 +1386,16 @@
       </x:c>
       <x:c r="B14" s="24"/>
       <x:c r="C14" s="26" t="str">
-        <x:v>Contabilidad auxiliar + Tributos y aportes</x:v>
+        <x:v>Factibilidad</x:v>
       </x:c>
       <x:c r="D14" s="26" t="str">
-        <x:v>36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 49, 57, 58, 59, 60, 61, 62, 92, 93</x:v>
+        <x:v>56, 104</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 49, 57, 58, 59, 60, 61, 62, 92, 93 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 56, 104 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F14" s="26" t="str">
-        <x:v>Conciliación y papeles de cierre · Calendario y conciliación fiscal auxiliar</x:v>
+        <x:v>Estudio de factibilidad y modelo</x:v>
       </x:c>
       <x:c r="G14" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1412,16 +1412,16 @@
       </x:c>
       <x:c r="B15" s="24"/>
       <x:c r="C15" s="26" t="str">
-        <x:v>Cumplimiento + Riesgos</x:v>
+        <x:v>Contabilidad auxiliar</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>29, 30, 31, 32, 33, 34, 35, 75, 76, 77, 78, 79, 80</x:v>
+        <x:v>36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 49, 92</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 29, 30, 31, 32, 33, 34, 35, 75, 76, 77, 78, 79, 80 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 49, 92 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F15" s="26" t="str">
-        <x:v>Matriz de aplicabilidad y plan · Mapa de riesgos y plan de tratamiento</x:v>
+        <x:v>Conciliación y papeles de cierre</x:v>
       </x:c>
       <x:c r="G15" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1438,16 +1438,16 @@
       </x:c>
       <x:c r="B16" s="24"/>
       <x:c r="C16" s="26" t="str">
-        <x:v>Indicadores</x:v>
+        <x:v>Tributos y aportes</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
-        <x:v>98, 99, 100, 101, 102, 103</x:v>
+        <x:v>57, 58, 59, 60, 61, 62, 93</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 98, 99, 100, 101, 102, 103 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 57, 58, 59, 60, 61, 62, 93 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F16" s="26" t="str">
-        <x:v>Fichas de indicadores y tablero</x:v>
+        <x:v>Calendario y conciliación fiscal auxiliar</x:v>
       </x:c>
       <x:c r="G16" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1464,16 +1464,16 @@
       </x:c>
       <x:c r="B17" s="24"/>
       <x:c r="C17" s="26" t="str">
-        <x:v>Seguimiento de proyectos + Compras y proveedores</x:v>
+        <x:v>Cumplimiento</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
-        <x:v>105, 106, 107, 108, 109, 110, 111, 112</x:v>
+        <x:v>29, 30, 31, 32, 33, 34, 35</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 105, 106, 107, 108, 109, 110, 111, 112 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 29, 30, 31, 32, 33, 34, 35 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F17" s="26" t="str">
-        <x:v>Informe físico-financiero y cronograma · Comparativo de ofertas y expediente</x:v>
+        <x:v>Matriz de aplicabilidad y plan</x:v>
       </x:c>
       <x:c r="G17" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1490,16 +1490,16 @@
       </x:c>
       <x:c r="B18" s="24"/>
       <x:c r="C18" s="26" t="str">
-        <x:v>Inventarios y activos + Procesos</x:v>
+        <x:v>Riesgos</x:v>
       </x:c>
       <x:c r="D18" s="26" t="str">
-        <x:v>113, 114, 115, 116</x:v>
+        <x:v>75, 76, 77, 78, 79, 80</x:v>
       </x:c>
       <x:c r="E18" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 113, 114, 115, 116 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 75, 76, 77, 78, 79, 80 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F18" s="26" t="str">
-        <x:v>Control de existencias y mantenimiento · Mapa de proceso y plan de mejora</x:v>
+        <x:v>Mapa de riesgos y plan de tratamiento</x:v>
       </x:c>
       <x:c r="G18" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1516,16 +1516,16 @@
       </x:c>
       <x:c r="B19" s="24"/>
       <x:c r="C19" s="26" t="str">
-        <x:v>Comercial y clientes</x:v>
+        <x:v>Indicadores + Seguimiento de proyectos</x:v>
       </x:c>
       <x:c r="D19" s="26" t="str">
-        <x:v>117, 118, 119, 120, 121, 122</x:v>
+        <x:v>98, 99, 100, 101, 102, 103, 105, 106, 107, 108, 109</x:v>
       </x:c>
       <x:c r="E19" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 117, 118, 119, 120, 121, 122 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 98, 99, 100, 101, 102, 103, 105, 106, 107, 108, 109 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F19" s="26" t="str">
-        <x:v>Propuesta comercial y seguimiento</x:v>
+        <x:v>Fichas de indicadores y tablero · Informe físico-financiero y cronograma</x:v>
       </x:c>
       <x:c r="G19" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1542,16 +1542,16 @@
       </x:c>
       <x:c r="B20" s="24"/>
       <x:c r="C20" s="26" t="str">
-        <x:v>Comunicación + Asistentes internos</x:v>
+        <x:v>Compras y proveedores + Inventarios y activos + Procesos</x:v>
       </x:c>
       <x:c r="D20" s="26" t="str">
-        <x:v>123, 124, 125, 126, 127, 128, 129, 130, 131, 132, 133, 134, 135, 136</x:v>
+        <x:v>110, 111, 112, 113, 114, 115, 116</x:v>
       </x:c>
       <x:c r="E20" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 123, 124, 125, 126, 127, 128, 129, 130, 131, 132, 133, 134, 135, 136 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 110, 111, 112, 113, 114, 115, 116 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F20" s="26" t="str">
-        <x:v>Contenido o guion multiformato · Asistente configurado y casos de prueba</x:v>
+        <x:v>Comparativo de ofertas y expediente · Control de existencias y mantenimiento · Mapa de proceso y plan de mejora</x:v>
       </x:c>
       <x:c r="G20" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1568,16 +1568,16 @@
       </x:c>
       <x:c r="B21" s="24"/>
       <x:c r="C21" s="26" t="str">
-        <x:v>Automatización + Diagnóstico e implantación</x:v>
+        <x:v>Comercial y clientes</x:v>
       </x:c>
       <x:c r="D21" s="26" t="str">
-        <x:v>137, 138, 139, 140, 141, 142, 143</x:v>
+        <x:v>117, 118, 119, 120, 121, 122</x:v>
       </x:c>
       <x:c r="E21" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 137, 138, 139, 140, 141, 142, 143 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 117, 118, 119, 120, 121, 122 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F21" s="26" t="str">
-        <x:v>Flujo, plantillas y procedimiento · Diagnóstico y hoja de ruta 30/60/90</x:v>
+        <x:v>Propuesta comercial y seguimiento</x:v>
       </x:c>
       <x:c r="G21" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1594,16 +1594,16 @@
       </x:c>
       <x:c r="B22" s="24"/>
       <x:c r="C22" s="26" t="str">
-        <x:v>Nuevos actores económicos + Reuniones y acuerdos</x:v>
+        <x:v>Comunicación</x:v>
       </x:c>
       <x:c r="D22" s="26" t="str">
-        <x:v>17, 18, 19, 20, 21, 22, 144</x:v>
+        <x:v>123, 124, 125, 126, 127, 128, 129</x:v>
       </x:c>
       <x:c r="E22" s="26" t="str">
-        <x:v>Diagnosticar, producir y actualizar los servicios 17, 18, 19, 20, 21, 22, 144 según contrato e insumos disponibles.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 123, 124, 125, 126, 127, 128, 129 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F22" s="26" t="str">
-        <x:v>Ruta de organización y expediente preparatorio · Agenda y seguimiento de tareas</x:v>
+        <x:v>Contenido o guion multiformato</x:v>
       </x:c>
       <x:c r="G22" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1620,16 +1620,16 @@
       </x:c>
       <x:c r="B23" s="24"/>
       <x:c r="C23" s="26" t="str">
-        <x:v>Control de calidad transversal</x:v>
+        <x:v>Asistentes internos + Automatización</x:v>
       </x:c>
       <x:c r="D23" s="26" t="str">
-        <x:v>Servicios contratados pendientes</x:v>
+        <x:v>130, 131, 132, 133, 134, 135, 136, 138, 139, 140</x:v>
       </x:c>
       <x:c r="E23" s="26" t="str">
-        <x:v>Revisar cifras, fuentes, vigencia y trazabilidad de todos los expedientes activos.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 130, 131, 132, 133, 134, 135, 136, 138, 139, 140 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F23" s="26" t="str">
-        <x:v>Registro de resultados, pendientes y evidencia</x:v>
+        <x:v>Asistente configurado y casos de prueba · Flujo, plantillas y procedimiento</x:v>
       </x:c>
       <x:c r="G23" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1646,16 +1646,16 @@
       </x:c>
       <x:c r="B24" s="24"/>
       <x:c r="C24" s="26" t="str">
-        <x:v>Entregas y aceptación</x:v>
+        <x:v>Diagnóstico e implantación + Nuevos actores económicos + Reuniones y acuerdos</x:v>
       </x:c>
       <x:c r="D24" s="26" t="str">
-        <x:v>Servicios contratados pendientes</x:v>
+        <x:v>17, 18, 19, 20, 21, 22, 137, 141, 142, 143, 144</x:v>
       </x:c>
       <x:c r="E24" s="26" t="str">
-        <x:v>Exportar entregables revisados; registrar acuses y aceptación del cliente.</x:v>
+        <x:v>Diagnosticar, producir y actualizar los servicios 17, 18, 19, 20, 21, 22, 137, 141, 142, 143, 144 según contrato e insumos disponibles.</x:v>
       </x:c>
       <x:c r="F24" s="26" t="str">
-        <x:v>Registro de resultados, pendientes y evidencia</x:v>
+        <x:v>Diagnóstico y hoja de ruta 30/60/90 · Ruta de organización y expediente preparatorio · Agenda y seguimiento de tareas</x:v>
       </x:c>
       <x:c r="G24" s="25" t="str">
         <x:v>Anotar archivo, fuente y revisión</x:v>
@@ -1672,13 +1672,13 @@
       </x:c>
       <x:c r="B25" s="24"/>
       <x:c r="C25" s="26" t="str">
-        <x:v>Informe y cierre</x:v>
+        <x:v>Calidad, entregas y aceptación</x:v>
       </x:c>
       <x:c r="D25" s="26" t="str">
         <x:v>Servicios contratados pendientes</x:v>
       </x:c>
       <x:c r="E25" s="26" t="str">
-        <x:v>Comparar lo contratado, lo entregado y lo aceptado; redactar informe de resultados reales.</x:v>
+        <x:v>Revisar cifras, fuentes y vigencia; exportar entregables revisados y registrar aceptación.</x:v>
       </x:c>
       <x:c r="F25" s="26" t="str">
         <x:v>Registro de resultados, pendientes y evidencia</x:v>
@@ -1698,13 +1698,13 @@
       </x:c>
       <x:c r="B26" s="24"/>
       <x:c r="C26" s="26" t="str">
-        <x:v>Replanificación y respaldo</x:v>
+        <x:v>Informe, replanificación y respaldo</x:v>
       </x:c>
       <x:c r="D26" s="26" t="str">
         <x:v>Servicios contratados pendientes</x:v>
       </x:c>
       <x:c r="E26" s="26" t="str">
-        <x:v>Acordar pendientes del mes siguiente, responsables y fechas; guardar respaldo.</x:v>
+        <x:v>Comparar lo contratado, entregado y aceptado; informar resultados reales, pendientes y respaldar.</x:v>
       </x:c>
       <x:c r="F26" s="26" t="str">
         <x:v>Registro de resultados, pendientes y evidencia</x:v>
@@ -2857,7 +2857,7 @@
         <x:v>Paquete previo de junta, agenda, preguntas y asuntos que requieren acuerdo.</x:v>
       </x:c>
       <x:c r="G23" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H23" s="29"/>
       <x:c r="I23" s="29"/>
@@ -2893,7 +2893,7 @@
         <x:v>Matriz de tareas y seguimiento; minutas y actas excluidas.</x:v>
       </x:c>
       <x:c r="G24" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H24" s="29"/>
       <x:c r="I24" s="29"/>
@@ -2929,7 +2929,7 @@
         <x:v>Registro de acuerdos, alertas y reporte de vencidos o bloqueados.</x:v>
       </x:c>
       <x:c r="G25" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H25" s="29"/>
       <x:c r="I25" s="29"/>
@@ -2965,7 +2965,7 @@
         <x:v>Informe de cumplimiento y lista de decisiones pendientes.</x:v>
       </x:c>
       <x:c r="G26" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H26" s="29"/>
       <x:c r="I26" s="29"/>
@@ -3001,7 +3001,7 @@
         <x:v>Presentación de cierre, informe de excepciones y propuesta de decisiones.</x:v>
       </x:c>
       <x:c r="G27" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H27" s="29"/>
       <x:c r="I27" s="29"/>
@@ -3037,7 +3037,7 @@
         <x:v>Índice de documentos aportados y matriz de seguimiento dentro del alcance autorizado.</x:v>
       </x:c>
       <x:c r="G28" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H28" s="29"/>
       <x:c r="I28" s="29"/>
@@ -3073,7 +3073,7 @@
         <x:v>Árbol de carpetas, índice maestro y norma de denominación.</x:v>
       </x:c>
       <x:c r="G29" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H29" s="29"/>
       <x:c r="I29" s="29"/>
@@ -3109,7 +3109,7 @@
         <x:v>Inventario clasificado y cola de excepciones.</x:v>
       </x:c>
       <x:c r="G30" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H30" s="29"/>
       <x:c r="I30" s="29"/>
@@ -3145,7 +3145,7 @@
         <x:v>Historial de versiones y relación de documentos oficiales.</x:v>
       </x:c>
       <x:c r="G31" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H31" s="29"/>
       <x:c r="I31" s="29"/>
@@ -3181,7 +3181,7 @@
         <x:v>Calendario de vencimientos y reporte de renovaciones.</x:v>
       </x:c>
       <x:c r="G32" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H32" s="29"/>
       <x:c r="I32" s="29"/>
@@ -3217,7 +3217,7 @@
         <x:v>Asistente de búsqueda con respuesta, fuente y fecha de revisión.</x:v>
       </x:c>
       <x:c r="G33" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H33" s="29"/>
       <x:c r="I33" s="29"/>
@@ -3253,7 +3253,7 @@
         <x:v>Base de conocimiento y programa de transferencia.</x:v>
       </x:c>
       <x:c r="G34" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H34" s="29"/>
       <x:c r="I34" s="29"/>
@@ -3289,7 +3289,7 @@
         <x:v>Boletín de cambios, ficha de fuente y alerta priorizada.</x:v>
       </x:c>
       <x:c r="G35" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H35" s="29"/>
       <x:c r="I35" s="29"/>
@@ -3325,7 +3325,7 @@
         <x:v>Resumen ejecutivo con referencias y preguntas abiertas.</x:v>
       </x:c>
       <x:c r="G36" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H36" s="29"/>
       <x:c r="I36" s="29"/>
@@ -3361,7 +3361,7 @@
         <x:v>Matriz de aplica, no aplica o requiere validación, con fundamento.</x:v>
       </x:c>
       <x:c r="G37" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H37" s="29"/>
       <x:c r="I37" s="29"/>
@@ -3397,7 +3397,7 @@
         <x:v>Plan de acciones con plazos y criterios de cierre.</x:v>
       </x:c>
       <x:c r="G38" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H38" s="29"/>
       <x:c r="I38" s="29"/>
@@ -3433,7 +3433,7 @@
         <x:v>Base de preguntas frecuentes revisada y lista para consulta.</x:v>
       </x:c>
       <x:c r="G39" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H39" s="29"/>
       <x:c r="I39" s="29"/>
@@ -3469,7 +3469,7 @@
         <x:v>Programa de actualización, materiales y registro de comprensión.</x:v>
       </x:c>
       <x:c r="G40" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H40" s="29"/>
       <x:c r="I40" s="29"/>
@@ -3505,7 +3505,7 @@
         <x:v>Mapa obligación a evidencia y lista de brechas.</x:v>
       </x:c>
       <x:c r="G41" s="3" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H41" s="29"/>
       <x:c r="I41" s="29"/>
@@ -3541,7 +3541,7 @@
         <x:v>Reporte de alertas, preguntas y acciones para el contador.</x:v>
       </x:c>
       <x:c r="G42" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H42" s="29"/>
       <x:c r="I42" s="29"/>
@@ -3577,7 +3577,7 @@
         <x:v>Listado de posibles errores con importe, fuente y motivo de alerta.</x:v>
       </x:c>
       <x:c r="G43" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H43" s="29"/>
       <x:c r="I43" s="29"/>
@@ -3613,7 +3613,7 @@
         <x:v>Lista de cierre, panel de avance y expediente final.</x:v>
       </x:c>
       <x:c r="G44" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H44" s="29"/>
       <x:c r="I44" s="29"/>
@@ -3649,7 +3649,7 @@
         <x:v>Estados parametrizados, cuentas sin mapear y comprobaciones.</x:v>
       </x:c>
       <x:c r="G45" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H45" s="29"/>
       <x:c r="I45" s="29"/>
@@ -3685,7 +3685,7 @@
         <x:v>Notas con cifras, explicación, política y fuente.</x:v>
       </x:c>
       <x:c r="G46" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H46" s="29"/>
       <x:c r="I46" s="29"/>
@@ -3721,7 +3721,7 @@
         <x:v>Matriz de variaciones, explicación solicitada y presentación ejecutiva.</x:v>
       </x:c>
       <x:c r="G47" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H47" s="29"/>
       <x:c r="I47" s="29"/>
@@ -3757,7 +3757,7 @@
         <x:v>Diferencias, antigüedad, responsable y plan de corrección.</x:v>
       </x:c>
       <x:c r="G48" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H48" s="29"/>
       <x:c r="I48" s="29"/>
@@ -3793,7 +3793,7 @@
         <x:v>Relación de registros sin soporte o con soporte insuficiente.</x:v>
       </x:c>
       <x:c r="G49" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H49" s="29"/>
       <x:c r="I49" s="29"/>
@@ -3829,7 +3829,7 @@
         <x:v>Diario bancario estructurado, resumen y operaciones por aclarar.</x:v>
       </x:c>
       <x:c r="G50" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H50" s="29"/>
       <x:c r="I50" s="29"/>
@@ -3865,7 +3865,7 @@
         <x:v>Conciliación, partidas pendientes y evidencia de revisión.</x:v>
       </x:c>
       <x:c r="G51" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H51" s="31"/>
       <x:c r="I51" s="31"/>
@@ -3901,7 +3901,7 @@
         <x:v>Alertas priorizadas y trazabilidad de las filas analizadas.</x:v>
       </x:c>
       <x:c r="G52" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H52" s="31"/>
       <x:c r="I52" s="31"/>
@@ -3937,7 +3937,7 @@
         <x:v>Parte diario para dirección y tesorería.</x:v>
       </x:c>
       <x:c r="G53" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H53" s="31"/>
       <x:c r="I53" s="31"/>
@@ -3973,7 +3973,7 @@
         <x:v>Flujo de caja proyectado y alertas de déficit o excedente.</x:v>
       </x:c>
       <x:c r="G54" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H54" s="31"/>
       <x:c r="I54" s="31"/>
@@ -4009,7 +4009,7 @@
         <x:v>Cadena de evidencia y explicación documentada.</x:v>
       </x:c>
       <x:c r="G55" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H55" s="31"/>
       <x:c r="I55" s="31"/>
@@ -4045,7 +4045,7 @@
         <x:v>Informe financiero, gráficos y decisiones sugeridas para análisis.</x:v>
       </x:c>
       <x:c r="G56" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H56" s="31"/>
       <x:c r="I56" s="31"/>
@@ -4081,7 +4081,7 @@
         <x:v>Presupuesto integrado, escenarios y notas de supuestos.</x:v>
       </x:c>
       <x:c r="G57" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H57" s="31"/>
       <x:c r="I57" s="31"/>
@@ -4117,7 +4117,7 @@
         <x:v>Reporte plan real, semáforos y medidas correctivas.</x:v>
       </x:c>
       <x:c r="G58" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H58" s="31"/>
       <x:c r="I58" s="31"/>
@@ -4153,7 +4153,7 @@
         <x:v>Ficha de costo, costo unitario y análisis de variación.</x:v>
       </x:c>
       <x:c r="G59" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H59" s="31"/>
       <x:c r="I59" s="31"/>
@@ -4189,7 +4189,7 @@
         <x:v>Ranking de rentabilidad y causas de pérdida o deterioro.</x:v>
       </x:c>
       <x:c r="G60" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H60" s="31"/>
       <x:c r="I60" s="31"/>
@@ -4225,7 +4225,7 @@
         <x:v>Escenarios base, conservador y exigente, con variables críticas.</x:v>
       </x:c>
       <x:c r="G61" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H61" s="31"/>
       <x:c r="I61" s="31"/>
@@ -4261,7 +4261,7 @@
         <x:v>Índice, documentos preparados, faltantes y resumen del proyecto.</x:v>
       </x:c>
       <x:c r="G62" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H62" s="31"/>
       <x:c r="I62" s="31"/>
@@ -4297,7 +4297,7 @@
         <x:v>Calendario y alertas previas.</x:v>
       </x:c>
       <x:c r="G63" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H63" s="31"/>
       <x:c r="I63" s="31"/>
@@ -4333,7 +4333,7 @@
         <x:v>Hoja de comprobación y lista de inconsistencias.</x:v>
       </x:c>
       <x:c r="G64" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H64" s="31"/>
       <x:c r="I64" s="31"/>
@@ -4369,7 +4369,7 @@
         <x:v>Conciliación, diferencias explicadas y acciones pendientes.</x:v>
       </x:c>
       <x:c r="G65" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H65" s="31"/>
       <x:c r="I65" s="31"/>
@@ -4405,7 +4405,7 @@
         <x:v>Paquete de trabajo y control de integridad.</x:v>
       </x:c>
       <x:c r="G66" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H66" s="31"/>
       <x:c r="I66" s="31"/>
@@ -4441,7 +4441,7 @@
         <x:v>Expediente de requerimiento y alertas de vencimiento.</x:v>
       </x:c>
       <x:c r="G67" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H67" s="31"/>
       <x:c r="I67" s="31"/>
@@ -4477,7 +4477,7 @@
         <x:v>Mapa de riesgos fiscales y plan preventivo.</x:v>
       </x:c>
       <x:c r="G68" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H68" s="31"/>
       <x:c r="I68" s="31"/>
@@ -4513,7 +4513,7 @@
         <x:v>Borrador contractual y ficha de datos pendientes.</x:v>
       </x:c>
       <x:c r="G69" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H69" s="31"/>
       <x:c r="I69" s="31"/>
@@ -4549,7 +4549,7 @@
         <x:v>Matriz de observaciones y propuesta de ajustes.</x:v>
       </x:c>
       <x:c r="G70" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H70" s="31"/>
       <x:c r="I70" s="31"/>
@@ -4585,7 +4585,7 @@
         <x:v>Ficha de contrato y calendario de obligaciones.</x:v>
       </x:c>
       <x:c r="G71" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H71" s="31"/>
       <x:c r="I71" s="31"/>
@@ -4621,7 +4621,7 @@
         <x:v>Panel contractual y expediente por contraparte.</x:v>
       </x:c>
       <x:c r="G72" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H72" s="31"/>
       <x:c r="I72" s="31"/>
@@ -4657,7 +4657,7 @@
         <x:v>Proyecto de reclamación o respuesta y expediente probatorio.</x:v>
       </x:c>
       <x:c r="G73" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H73" s="31"/>
       <x:c r="I73" s="31"/>
@@ -4693,7 +4693,7 @@
         <x:v>Resumen preparatorio y relación de evidencias para revisión profesional.</x:v>
       </x:c>
       <x:c r="G74" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H74" s="31"/>
       <x:c r="I74" s="31"/>
@@ -4729,7 +4729,7 @@
         <x:v>Informe diagnóstico, matriz de brechas y prioridades.</x:v>
       </x:c>
       <x:c r="G75" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H75" s="31"/>
       <x:c r="I75" s="31"/>
@@ -4765,7 +4765,7 @@
         <x:v>Matriz riesgo control responsable evidencia.</x:v>
       </x:c>
       <x:c r="G76" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H76" s="31"/>
       <x:c r="I76" s="31"/>
@@ -4801,7 +4801,7 @@
         <x:v>Panel de autoevaluación y lista de excepciones.</x:v>
       </x:c>
       <x:c r="G77" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H77" s="31"/>
       <x:c r="I77" s="31"/>
@@ -4837,7 +4837,7 @@
         <x:v>Plan de medidas y tablero de seguimiento.</x:v>
       </x:c>
       <x:c r="G78" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H78" s="31"/>
       <x:c r="I78" s="31"/>
@@ -4873,7 +4873,7 @@
         <x:v>Reporte de medidas vencidas, bloqueadas o cerradas.</x:v>
       </x:c>
       <x:c r="G79" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H79" s="31"/>
       <x:c r="I79" s="31"/>
@@ -4909,7 +4909,7 @@
         <x:v>Papeles de trabajo y resumen de hallazgos.</x:v>
       </x:c>
       <x:c r="G80" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H80" s="31"/>
       <x:c r="I80" s="31"/>
@@ -4945,7 +4945,7 @@
         <x:v>Registro priorizado y mapa de calor.</x:v>
       </x:c>
       <x:c r="G81" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H81" s="31"/>
       <x:c r="I81" s="31"/>
@@ -4981,7 +4981,7 @@
         <x:v>Informe periódico de riesgos y decisiones requeridas.</x:v>
       </x:c>
       <x:c r="G82" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H82" s="31"/>
       <x:c r="I82" s="31"/>
@@ -5017,7 +5017,7 @@
         <x:v>Informe de incidente y plan de investigación.</x:v>
       </x:c>
       <x:c r="G83" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H83" s="31"/>
       <x:c r="I83" s="31"/>
@@ -5053,7 +5053,7 @@
         <x:v>Plan de continuidad y ejercicios de prueba.</x:v>
       </x:c>
       <x:c r="G84" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H84" s="31"/>
       <x:c r="I84" s="31"/>
@@ -5089,7 +5089,7 @@
         <x:v>Alertas con umbral, responsable y acción esperada.</x:v>
       </x:c>
       <x:c r="G85" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H85" s="31"/>
       <x:c r="I85" s="31"/>
@@ -5125,7 +5125,7 @@
         <x:v>Informe ejecutivo y presentación.</x:v>
       </x:c>
       <x:c r="G86" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H86" s="31"/>
       <x:c r="I86" s="31"/>
@@ -5161,7 +5161,7 @@
         <x:v>Diagnóstico de preparación y plan de cierre de brechas.</x:v>
       </x:c>
       <x:c r="G87" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H87" s="31"/>
       <x:c r="I87" s="31"/>
@@ -5197,7 +5197,7 @@
         <x:v>Expediente indexado y cronología.</x:v>
       </x:c>
       <x:c r="G88" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H88" s="31"/>
       <x:c r="I88" s="31"/>
@@ -5233,7 +5233,7 @@
         <x:v>Protocolo, bitácora y lista de contactos.</x:v>
       </x:c>
       <x:c r="G89" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H89" s="31"/>
       <x:c r="I89" s="31"/>
@@ -5269,7 +5269,7 @@
         <x:v>Bitácora de entrega y copia de respaldo.</x:v>
       </x:c>
       <x:c r="G90" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H90" s="31"/>
       <x:c r="I90" s="31"/>
@@ -5305,7 +5305,7 @@
         <x:v>Ficha de hallazgo y ruta de decisión.</x:v>
       </x:c>
       <x:c r="G91" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H91" s="31"/>
       <x:c r="I91" s="31"/>
@@ -5341,7 +5341,7 @@
         <x:v>Borrador y expediente de anexos.</x:v>
       </x:c>
       <x:c r="G92" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H92" s="31"/>
       <x:c r="I92" s="31"/>
@@ -5377,7 +5377,7 @@
         <x:v>Panel posauditoría e informe de cierre.</x:v>
       </x:c>
       <x:c r="G93" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H93" s="31"/>
       <x:c r="I93" s="31"/>
@@ -5413,7 +5413,7 @@
         <x:v>Índice por trabajador y lista de documentos faltantes o vencidos.</x:v>
       </x:c>
       <x:c r="G94" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H94" s="31"/>
       <x:c r="I94" s="31"/>
@@ -5449,7 +5449,7 @@
         <x:v>Borrador, anexos y control de aprobación.</x:v>
       </x:c>
       <x:c r="G95" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H95" s="31"/>
       <x:c r="I95" s="31"/>
@@ -5485,7 +5485,7 @@
         <x:v>Lista de tareas y expediente de movimiento.</x:v>
       </x:c>
       <x:c r="G96" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H96" s="31"/>
       <x:c r="I96" s="31"/>
@@ -5521,7 +5521,7 @@
         <x:v>Resumen por persona y área, excepciones y próximos vencimientos.</x:v>
       </x:c>
       <x:c r="G97" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H97" s="31"/>
       <x:c r="I97" s="31"/>
@@ -5557,7 +5557,7 @@
         <x:v>Reporte de excepciones antes del pago.</x:v>
       </x:c>
       <x:c r="G98" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H98" s="31"/>
       <x:c r="I98" s="31"/>
@@ -5593,7 +5593,7 @@
         <x:v>Conciliación y calendario de obligaciones.</x:v>
       </x:c>
       <x:c r="G99" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H99" s="31"/>
       <x:c r="I99" s="31"/>
@@ -5629,7 +5629,7 @@
         <x:v>Matriz de competencias y programa de capacitación.</x:v>
       </x:c>
       <x:c r="G100" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H100" s="31"/>
       <x:c r="I100" s="31"/>
@@ -5665,7 +5665,7 @@
         <x:v>Evaluación estructurada y plan individual.</x:v>
       </x:c>
       <x:c r="G101" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H101" s="31"/>
       <x:c r="I101" s="31"/>
@@ -5701,7 +5701,7 @@
         <x:v>Expediente de SST, alertas y plan preventivo.</x:v>
       </x:c>
       <x:c r="G102" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H102" s="31"/>
       <x:c r="I102" s="31"/>
@@ -5737,7 +5737,7 @@
         <x:v>Panel mensual y explicación de variaciones.</x:v>
       </x:c>
       <x:c r="G103" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H103" s="31"/>
       <x:c r="I103" s="31"/>
@@ -5773,7 +5773,7 @@
         <x:v>Ficha técnica de cada indicador.</x:v>
       </x:c>
       <x:c r="G104" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H104" s="31"/>
       <x:c r="I104" s="31"/>
@@ -5809,7 +5809,7 @@
         <x:v>Base consolidada y reporte de calidad.</x:v>
       </x:c>
       <x:c r="G105" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H105" s="31"/>
       <x:c r="I105" s="31"/>
@@ -5845,7 +5845,7 @@
         <x:v>Panel con tendencia, meta, semáforo y explicación.</x:v>
       </x:c>
       <x:c r="G106" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H106" s="31"/>
       <x:c r="I106" s="31"/>
@@ -5881,7 +5881,7 @@
         <x:v>Informe estadístico y gráficos.</x:v>
       </x:c>
       <x:c r="G107" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H107" s="31"/>
       <x:c r="I107" s="31"/>
@@ -5917,7 +5917,7 @@
         <x:v>Paquete estadístico listo para revisión y presentación autorizada.</x:v>
       </x:c>
       <x:c r="G108" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H108" s="31"/>
       <x:c r="I108" s="31"/>
@@ -5953,7 +5953,7 @@
         <x:v>Informe de errores y base depurada para aprobación.</x:v>
       </x:c>
       <x:c r="G109" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H109" s="31"/>
       <x:c r="I109" s="31"/>
@@ -5989,7 +5989,7 @@
         <x:v>Ficha de proyecto y expediente para revisión.</x:v>
       </x:c>
       <x:c r="G110" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H110" s="31"/>
       <x:c r="I110" s="31"/>
@@ -6025,7 +6025,7 @@
         <x:v>Tablero físico financiero y lista de desviaciones.</x:v>
       </x:c>
       <x:c r="G111" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H111" s="31"/>
       <x:c r="I111" s="31"/>
@@ -6061,7 +6061,7 @@
         <x:v>Cronograma actualizado y alertas de retraso.</x:v>
       </x:c>
       <x:c r="G112" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H112" s="31"/>
       <x:c r="I112" s="31"/>
@@ -6097,7 +6097,7 @@
         <x:v>Informe presupuestario y alertas de desviación.</x:v>
       </x:c>
       <x:c r="G113" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H113" s="31"/>
       <x:c r="I113" s="31"/>
@@ -6133,7 +6133,7 @@
         <x:v>Informe técnico financiero y presentación.</x:v>
       </x:c>
       <x:c r="G114" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H114" s="31"/>
       <x:c r="I114" s="31"/>
@@ -6169,7 +6169,7 @@
         <x:v>Expediente de cierre y evaluación final.</x:v>
       </x:c>
       <x:c r="G115" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H115" s="31"/>
       <x:c r="I115" s="31"/>
@@ -6205,7 +6205,7 @@
         <x:v>Solicitud completa y flujo de aprobación.</x:v>
       </x:c>
       <x:c r="G116" t="n">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H116" s="31"/>
       <x:c r="I116" s="31"/>
@@ -6241,7 +6241,7 @@
         <x:v>Matriz comparativa y preguntas para decisión.</x:v>
       </x:c>
       <x:c r="G117" t="n">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H117" s="31"/>
       <x:c r="I117" s="31"/>
@@ -6277,7 +6277,7 @@
         <x:v>Ficha de proveedor y alertas.</x:v>
       </x:c>
       <x:c r="G118" t="n">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H118" s="31"/>
       <x:c r="I118" s="31"/>
@@ -6313,7 +6313,7 @@
         <x:v>Reporte de inventario y acciones priorizadas.</x:v>
       </x:c>
       <x:c r="G119" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H119" s="31"/>
       <x:c r="I119" s="31"/>
@@ -6349,7 +6349,7 @@
         <x:v>Registro de activos, alertas y conciliación física.</x:v>
       </x:c>
       <x:c r="G120" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H120" s="31"/>
       <x:c r="I120" s="31"/>
@@ -6385,7 +6385,7 @@
         <x:v>Calendario de mantenimiento y alertas.</x:v>
       </x:c>
       <x:c r="G121" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H121" s="31"/>
       <x:c r="I121" s="31"/>
@@ -6421,7 +6421,7 @@
         <x:v>Mapa del proceso, línea base y oportunidades de automatización.</x:v>
       </x:c>
       <x:c r="G122" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H122" s="31"/>
       <x:c r="I122" s="31"/>
@@ -6457,7 +6457,7 @@
         <x:v>Embudo comercial y recordatorios.</x:v>
       </x:c>
       <x:c r="G123" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H123" s="31"/>
       <x:c r="I123" s="31"/>
@@ -6493,7 +6493,7 @@
         <x:v>Propuesta profesional y resumen para presentación.</x:v>
       </x:c>
       <x:c r="G124" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H124" s="31"/>
       <x:c r="I124" s="31"/>
@@ -6529,7 +6529,7 @@
         <x:v>Ficha de costo, precio y límites del servicio.</x:v>
       </x:c>
       <x:c r="G125" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H125" s="31"/>
       <x:c r="I125" s="31"/>
@@ -6565,7 +6565,7 @@
         <x:v>Panel de clientes y reporte de atención.</x:v>
       </x:c>
       <x:c r="G126" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H126" s="31"/>
       <x:c r="I126" s="31"/>
@@ -6601,7 +6601,7 @@
         <x:v>Resumen de reclamaciones y plan de mejora.</x:v>
       </x:c>
       <x:c r="G127" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H127" s="31"/>
       <x:c r="I127" s="31"/>
@@ -6637,7 +6637,7 @@
         <x:v>Informe de percepción y acciones.</x:v>
       </x:c>
       <x:c r="G128" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H128" s="31"/>
       <x:c r="I128" s="31"/>
@@ -6673,7 +6673,7 @@
         <x:v>Presentación editable y guion del expositor.</x:v>
       </x:c>
       <x:c r="G129" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H129" s="31"/>
       <x:c r="I129" s="31"/>
@@ -6709,7 +6709,7 @@
         <x:v>Video y resumen escrito.</x:v>
       </x:c>
       <x:c r="G130" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H130" s="31"/>
       <x:c r="I130" s="31"/>
@@ -6745,7 +6745,7 @@
         <x:v>Audio o guion, ficha de fuentes y puntos clave.</x:v>
       </x:c>
       <x:c r="G131" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H131" s="31"/>
       <x:c r="I131" s="31"/>
@@ -6781,7 +6781,7 @@
         <x:v>Boletín listo para distribuir.</x:v>
       </x:c>
       <x:c r="G132" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H132" s="31"/>
       <x:c r="I132" s="31"/>
@@ -6817,7 +6817,7 @@
         <x:v>Paquete formativo por rol.</x:v>
       </x:c>
       <x:c r="G133" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H133" s="31"/>
       <x:c r="I133" s="31"/>
@@ -6853,7 +6853,7 @@
         <x:v>Guion y tarjeta de mensajes.</x:v>
       </x:c>
       <x:c r="G134" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H134" s="31"/>
       <x:c r="I134" s="31"/>
@@ -6889,7 +6889,7 @@
         <x:v>Paquete de contenidos coherentes.</x:v>
       </x:c>
       <x:c r="G135" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H135" s="31"/>
       <x:c r="I135" s="31"/>
@@ -6925,7 +6925,7 @@
         <x:v>Asistente con respuesta, fuente, versión y escalamiento.</x:v>
       </x:c>
       <x:c r="G136" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H136" s="31"/>
       <x:c r="I136" s="31"/>
@@ -6961,7 +6961,7 @@
         <x:v>Resumen diario o semanal y lista de prioridades.</x:v>
       </x:c>
       <x:c r="G137" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H137" s="31"/>
       <x:c r="I137" s="31"/>
@@ -6997,7 +6997,7 @@
         <x:v>Consulta documentada y papeles de trabajo.</x:v>
       </x:c>
       <x:c r="G138" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H138" s="31"/>
       <x:c r="I138" s="31"/>
@@ -7033,7 +7033,7 @@
         <x:v>Respuesta con fuentes y acciones pendientes.</x:v>
       </x:c>
       <x:c r="G139" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H139" s="31"/>
       <x:c r="I139" s="31"/>
@@ -7069,7 +7069,7 @@
         <x:v>Cola de cambios y borrador de impacto.</x:v>
       </x:c>
       <x:c r="G140" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H140" s="31"/>
       <x:c r="I140" s="31"/>
@@ -7105,7 +7105,7 @@
         <x:v>Panel actualizado y excepciones.</x:v>
       </x:c>
       <x:c r="G141" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H141" s="31"/>
       <x:c r="I141" s="31"/>
@@ -7141,7 +7141,7 @@
         <x:v>Expediente único y salida integrada.</x:v>
       </x:c>
       <x:c r="G142" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H142" s="31"/>
       <x:c r="I142" s="31"/>
@@ -7177,7 +7177,7 @@
         <x:v>Mapa de situación, brechas y prioridades.</x:v>
       </x:c>
       <x:c r="G143" t="n">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H143" s="31"/>
       <x:c r="I143" s="31"/>
@@ -7213,7 +7213,7 @@
         <x:v>Catálogo de tareas y puntuación de automatización.</x:v>
       </x:c>
       <x:c r="G144" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H144" s="31"/>
       <x:c r="I144" s="31"/>
@@ -7249,7 +7249,7 @@
         <x:v>Informe de ahorro, capacidad liberada y calidad.</x:v>
       </x:c>
       <x:c r="G145" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H145" s="31"/>
       <x:c r="I145" s="31"/>
@@ -7285,7 +7285,7 @@
         <x:v>Piloto operativo, manual y criterio de aceptación.</x:v>
       </x:c>
       <x:c r="G146" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H146" s="31"/>
       <x:c r="I146" s="31"/>
@@ -7321,7 +7321,7 @@
         <x:v>Sistema de trabajo listo para operar.</x:v>
       </x:c>
       <x:c r="G147" t="n">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H147" s="31"/>
       <x:c r="I147" s="31"/>
@@ -7357,7 +7357,7 @@
         <x:v>Entregables aprobados, panel, expediente y soporte.</x:v>
       </x:c>
       <x:c r="G148" t="n">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H148" s="31"/>
       <x:c r="I148" s="31"/>
@@ -7393,7 +7393,7 @@
         <x:v>Sistema transferido, manuales, evaluación y soporte.</x:v>
       </x:c>
       <x:c r="G149" t="n">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H149" s="31"/>
       <x:c r="I149" s="31"/>
@@ -7429,7 +7429,7 @@
         <x:v>Ruta de organización y expediente preparatorio</x:v>
       </x:c>
       <x:c r="G150" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H150" s="31"/>
       <x:c r="I150" s="31"/>
@@ -7475,7 +7475,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3760128187d646f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ed601723e79492a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>